<commit_message>
update lectures 4 and 5
</commit_message>
<xml_diff>
--- a/schedule2025.xlsx
+++ b/schedule2025.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9d9648ccaee313cb/Documents/DataHandling/datahandling-lecture/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{98FDF52C-1B09-43C0-B0DA-78556B5A21F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6F72218-71C6-4812-B371-9FAF361549D8}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{98FDF52C-1B09-43C0-B0DA-78556B5A21F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD892061-33FB-4131-9E5F-EC4D72C165F7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1_2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="64">
   <si>
     <t>Date</t>
   </si>
@@ -78,9 +78,6 @@
     <t>An introduction to data and data processing</t>
   </si>
   <si>
-    <t>Data storage and data structures</t>
-  </si>
-  <si>
     <t>Exercises/Workshop 2: Data storage and data structures</t>
   </si>
   <si>
@@ -126,9 +123,6 @@
     <t>Federica Mascolo</t>
   </si>
   <si>
-    <t>Rectangular data</t>
-  </si>
-  <si>
     <t>Visualisation</t>
   </si>
   <si>
@@ -138,9 +132,6 @@
     <t>Summary, Wrap-up, Final workshop</t>
   </si>
   <si>
-    <t>Non-rectangular data. Guest spot: Minna Heim</t>
-  </si>
-  <si>
     <t>Analytics, more visualisation, and data products</t>
   </si>
   <si>
@@ -207,12 +198,6 @@
     <t>DataHandlingPocketReference chapter 3, R4DS chapter 1, Mu chapter 2.</t>
   </si>
   <si>
-    <t>DataHandlingPocketReference chapter 4, Mu chapter 5.1-5.4</t>
-  </si>
-  <si>
-    <t>DataHandlingPocketReference chapter 8.1-8.4, Mu chapter 9.7</t>
-  </si>
-  <si>
     <t>DataHandlingPocketReference chapter 5-7, 8.5, R4DS chapter 7; Mu chapter 5.5, Webb et al. (2020), Gentzkow et al. (2019)</t>
   </si>
   <si>
@@ -220,6 +205,18 @@
   </si>
   <si>
     <t>DataHandlingPocketReference chapters 10-11</t>
+  </si>
+  <si>
+    <t>From text to data: data structures and rectangular data</t>
+  </si>
+  <si>
+    <t>DataHandlingPocketReference chapter 4, Mu chapter 5.1-5.4; DataHandlingPocketReference chapter 8.1-8.4, Mu chapter 9.7</t>
+  </si>
+  <si>
+    <t>Nonrectangular data</t>
+  </si>
+  <si>
+    <t>Retrieving data from the web: API</t>
   </si>
 </sst>
 </file>
@@ -1571,7 +1568,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>7</v>
@@ -1586,15 +1583,15 @@
         <v>10</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="26" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B3" s="27" t="s">
         <v>13</v>
@@ -1603,19 +1600,19 @@
         <v>14</v>
       </c>
       <c r="D3" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="F3" s="29" t="s">
         <v>31</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>32</v>
       </c>
       <c r="G3" s="29"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>7</v>
@@ -1633,12 +1630,12 @@
         <v>12</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -1656,12 +1653,12 @@
         <v>12</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>13</v>
@@ -1673,16 +1670,16 @@
         <v>15</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G6" s="12"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>7</v>
@@ -1694,18 +1691,18 @@
         <v>9</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>7</v>
@@ -1717,18 +1714,18 @@
         <v>9</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>7</v>
@@ -1740,18 +1737,16 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>62</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="G9" s="7"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>13</v>
@@ -1763,42 +1758,42 @@
         <v>15</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G10" s="12"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
       <c r="D11" s="15"/>
       <c r="E11" s="16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F11" s="17"/>
       <c r="G11" s="17"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="15"/>
       <c r="E12" s="16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F12" s="17"/>
       <c r="G12" s="17"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>7</v>
@@ -1810,18 +1805,18 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>7</v>
@@ -1833,18 +1828,18 @@
         <v>9</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>13</v>
@@ -1856,16 +1851,16 @@
         <v>15</v>
       </c>
       <c r="E15" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="12" t="s">
         <v>23</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>24</v>
       </c>
       <c r="G15" s="12"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="22" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B16" s="23" t="s">
         <v>7</v>
@@ -1877,16 +1872,16 @@
         <v>9</v>
       </c>
       <c r="E16" s="25" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G16" s="25"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="30" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B17" s="31" t="s">
         <v>7</v>
@@ -1898,18 +1893,18 @@
         <v>9</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F17" s="33" t="s">
         <v>12</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>13</v>
@@ -1921,16 +1916,16 @@
         <v>15</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G18" s="12"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>7</v>
@@ -1942,18 +1937,18 @@
         <v>9</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="34" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B20" s="35" t="s">
         <v>7</v>
@@ -1965,7 +1960,7 @@
         <v>9</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F20" s="38" t="s">
         <v>12</v>
@@ -1974,7 +1969,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>7</v>
@@ -1986,7 +1981,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>12</v>
@@ -1994,7 +1989,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>13</v>
@@ -2006,16 +2001,16 @@
         <v>15</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G22" s="12"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B23" s="18" t="s">
         <v>13</v>
@@ -2024,10 +2019,10 @@
         <v>14</v>
       </c>
       <c r="D23" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23" s="21" t="s">
         <v>27</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>28</v>
       </c>
       <c r="F23" s="21" t="s">
         <v>12</v>

</xml_diff>